<commit_message>
feat: No trade energy storage
</commit_message>
<xml_diff>
--- a/datasets/test.xlsx
+++ b/datasets/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\info\IV-1\licenta\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487987BF-6D10-444D-861F-4A05A58CEFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CFB69B3-67AB-4A9D-B84C-91F95B7F44BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3312" yWindow="3312" windowWidth="17280" windowHeight="8964" activeTab="2" xr2:uid="{0739AF66-2B1F-496E-9647-EADDFB9C2716}"/>
+    <workbookView xWindow="3312" yWindow="3312" windowWidth="17280" windowHeight="8964" xr2:uid="{0739AF66-2B1F-496E-9647-EADDFB9C2716}"/>
   </bookViews>
   <sheets>
     <sheet name="MG stats" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t>consume</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>discharge_efficiency</t>
+  </si>
+  <si>
+    <t>initial_stored_energy</t>
   </si>
 </sst>
 </file>
@@ -399,14 +402,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188723D3-3345-47D9-AD7F-A291F6E3188C}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.21875" customWidth="1"/>
     <col min="3" max="3" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -416,8 +419,11 @@
       <c r="C1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -427,8 +433,11 @@
       <c r="C2">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -437,6 +446,9 @@
       </c>
       <c r="C3">
         <v>0.4</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rounding characteristics + some tests
</commit_message>
<xml_diff>
--- a/datasets/test.xlsx
+++ b/datasets/test.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\info\IV-1\licenta\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B61019F3-2571-4FAE-8182-894154BC3D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8C6A4A-3178-4533-A81A-CD6228EA7FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3312" yWindow="3312" windowWidth="17280" windowHeight="8964" xr2:uid="{0739AF66-2B1F-496E-9647-EADDFB9C2716}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0739AF66-2B1F-496E-9647-EADDFB9C2716}"/>
   </bookViews>
   <sheets>
     <sheet name="MG stats" sheetId="2" r:id="rId1"/>
     <sheet name="MG1" sheetId="1" r:id="rId2"/>
     <sheet name="MG2" sheetId="3" r:id="rId3"/>
     <sheet name="MG3" sheetId="4" r:id="rId4"/>
+    <sheet name="MG4" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
   <si>
     <t>consume</t>
   </si>
@@ -58,6 +59,9 @@
   </si>
   <si>
     <t>MG3</t>
+  </si>
+  <si>
+    <t>MG4</t>
   </si>
 </sst>
 </file>
@@ -409,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{188723D3-3345-47D9-AD7F-A291F6E3188C}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.21875" customWidth="1"/>
@@ -482,6 +486,23 @@
       </c>
       <c r="E4">
         <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -757,4 +778,94 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C45F896-58EF-407A-AACD-CC57B176B875}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>0</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>0</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>